<commit_message>
Deploying to master from  @ ee147728731deb44e6b8faea08873046c8746793 🚀
</commit_message>
<xml_diff>
--- a/assets/excel/2025_4-1-2.xlsx
+++ b/assets/excel/2025_4-1-2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Hannover\Dez15_Uebergreifende_Analysen\Projekte\Integrationsmonitoring\github\MT_Site\assets\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Hannover\Dez15_Uebergreifende_Analysen\Projekte\Integrationsmonitoring\Schlesier\MT_Site\assets\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F9154A6C-4695-403B-8373-C9E26676EC0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B1D7603-0B72-41B7-B8A4-2738AD2F5865}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{18F03383-72E2-4C81-906D-6A02646D6F2E}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{18F03383-72E2-4C81-906D-6A02646D6F2E}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -147,13 +147,13 @@
     <t>Niedersächsisches Ministerium für Soziales, Gesundheit und Gleichstellung (Hrsg.),</t>
   </si>
   <si>
-    <t>© Landesamt für Statistik Niedersachsen, Hannover 2025,</t>
-  </si>
-  <si>
     <t>Vervielfältigung und Verbreitung, auch auszugsweise, mit Quellenangabe gestattet.</t>
   </si>
   <si>
     <t>https://www.integrationsmonitoring.niedersachsen.de</t>
+  </si>
+  <si>
+    <t>© Landesamt für Statistik Niedersachsen, Hannover 2026,</t>
   </si>
 </sst>
 </file>
@@ -418,36 +418,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -589,6 +559,36 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -954,2117 +954,2117 @@
       <c r="F6" s="5"/>
     </row>
     <row r="7" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="62" t="s">
         <v>4</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="62" t="s">
         <v>5</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="62" t="s">
         <v>6</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="F7" s="65" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="8" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="10"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="13"/>
+      <c r="B8" s="60"/>
+      <c r="C8" s="63"/>
+      <c r="D8" s="64"/>
+      <c r="E8" s="64"/>
+      <c r="F8" s="66"/>
     </row>
     <row r="9" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="14"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="15" t="s">
+      <c r="B9" s="61"/>
+      <c r="C9" s="64"/>
+      <c r="D9" s="67" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="16"/>
-      <c r="F9" s="16"/>
-      <c r="L9" s="17" t="s">
+      <c r="E9" s="68"/>
+      <c r="F9" s="68"/>
+      <c r="L9" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="M9" s="17" t="s">
+      <c r="M9" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="N9" s="17" t="s">
+      <c r="N9" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="O9" s="17" t="s">
+      <c r="O9" s="7" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="10" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="E10" s="19" t="s">
+      <c r="E10" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F10" s="19" t="s">
+      <c r="F10" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="2:15" s="61" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="62" t="s">
+    <row r="11" spans="2:15" s="51" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="52" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="63">
+      <c r="C11" s="53">
         <v>2024</v>
       </c>
-      <c r="D11" s="64">
+      <c r="D11" s="54">
         <v>24726</v>
       </c>
-      <c r="E11" s="64">
+      <c r="E11" s="54">
         <v>24079</v>
       </c>
-      <c r="F11" s="64">
+      <c r="F11" s="54">
         <v>647</v>
       </c>
     </row>
-    <row r="12" spans="2:15" s="61" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="62" t="s">
+    <row r="12" spans="2:15" s="51" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="52" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="63">
+      <c r="C12" s="53">
         <v>2024</v>
       </c>
-      <c r="D12" s="64">
+      <c r="D12" s="54">
         <v>3077</v>
       </c>
-      <c r="E12" s="64">
+      <c r="E12" s="54">
         <v>2798</v>
       </c>
-      <c r="F12" s="64">
+      <c r="F12" s="54">
         <v>279</v>
       </c>
     </row>
-    <row r="13" spans="2:15" s="61" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="62" t="s">
+    <row r="13" spans="2:15" s="51" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="52" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="63">
+      <c r="C13" s="53">
         <v>2024</v>
       </c>
-      <c r="D13" s="64">
+      <c r="D13" s="54">
         <v>33422</v>
       </c>
-      <c r="E13" s="64">
+      <c r="E13" s="54">
         <v>29617</v>
       </c>
-      <c r="F13" s="64">
+      <c r="F13" s="54">
         <v>3805</v>
       </c>
     </row>
-    <row r="14" spans="2:15" s="61" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="62" t="s">
+    <row r="14" spans="2:15" s="51" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="52" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="63">
+      <c r="C14" s="53">
         <v>2024</v>
       </c>
-      <c r="D14" s="64">
+      <c r="D14" s="54">
         <v>11381</v>
       </c>
-      <c r="E14" s="64">
+      <c r="E14" s="54">
         <v>8966</v>
       </c>
-      <c r="F14" s="64">
+      <c r="F14" s="54">
         <v>2415</v>
       </c>
     </row>
-    <row r="15" spans="2:15" s="61" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="62" t="s">
+    <row r="15" spans="2:15" s="51" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="52" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="63">
+      <c r="C15" s="53">
         <v>2024</v>
       </c>
-      <c r="D15" s="64">
+      <c r="D15" s="54">
         <v>2446</v>
       </c>
-      <c r="E15" s="64">
+      <c r="E15" s="54">
         <v>1897</v>
       </c>
-      <c r="F15" s="64">
+      <c r="F15" s="54">
         <v>549</v>
       </c>
     </row>
-    <row r="16" spans="2:15" s="61" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="62" t="s">
+    <row r="16" spans="2:15" s="51" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="52" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="63">
+      <c r="C16" s="53">
         <v>2024</v>
       </c>
-      <c r="D16" s="64">
+      <c r="D16" s="54">
         <v>4437</v>
       </c>
-      <c r="E16" s="64">
+      <c r="E16" s="54">
         <v>2237</v>
       </c>
-      <c r="F16" s="64">
+      <c r="F16" s="54">
         <v>2200</v>
       </c>
     </row>
-    <row r="17" spans="2:6" s="68" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="65" t="s">
+    <row r="17" spans="2:6" s="58" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="55" t="s">
         <v>5</v>
       </c>
-      <c r="C17" s="66">
+      <c r="C17" s="56">
         <v>2024</v>
       </c>
-      <c r="D17" s="67">
+      <c r="D17" s="57">
         <v>79489</v>
       </c>
-      <c r="E17" s="67">
+      <c r="E17" s="57">
         <v>69594</v>
       </c>
-      <c r="F17" s="67">
+      <c r="F17" s="57">
         <v>9895</v>
       </c>
     </row>
     <row r="18" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="20" t="s">
+      <c r="B18" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C18" s="23">
+      <c r="C18" s="13">
         <v>2023</v>
       </c>
-      <c r="D18" s="24">
+      <c r="D18" s="14">
         <v>24790</v>
       </c>
-      <c r="E18" s="24">
+      <c r="E18" s="14">
         <v>23949</v>
       </c>
-      <c r="F18" s="24">
+      <c r="F18" s="14">
         <v>841</v>
       </c>
     </row>
     <row r="19" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="20" t="s">
+      <c r="B19" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C19" s="23">
+      <c r="C19" s="13">
         <v>2023</v>
       </c>
-      <c r="D19" s="24">
+      <c r="D19" s="14">
         <v>2816</v>
       </c>
-      <c r="E19" s="24">
+      <c r="E19" s="14">
         <v>2592</v>
       </c>
-      <c r="F19" s="24">
+      <c r="F19" s="14">
         <v>224</v>
       </c>
     </row>
     <row r="20" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="20" t="s">
+      <c r="B20" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C20" s="23">
+      <c r="C20" s="13">
         <v>2023</v>
       </c>
-      <c r="D20" s="24">
+      <c r="D20" s="14">
         <v>32696</v>
       </c>
-      <c r="E20" s="24">
+      <c r="E20" s="14">
         <v>29226</v>
       </c>
-      <c r="F20" s="24">
+      <c r="F20" s="14">
         <v>3470</v>
       </c>
     </row>
     <row r="21" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="20" t="s">
+      <c r="B21" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C21" s="23">
+      <c r="C21" s="13">
         <v>2023</v>
       </c>
-      <c r="D21" s="24">
+      <c r="D21" s="14">
         <v>10659</v>
       </c>
-      <c r="E21" s="24">
+      <c r="E21" s="14">
         <v>8628</v>
       </c>
-      <c r="F21" s="24">
+      <c r="F21" s="14">
         <v>2031</v>
       </c>
     </row>
     <row r="22" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="20" t="s">
+      <c r="B22" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C22" s="23">
+      <c r="C22" s="13">
         <v>2023</v>
       </c>
-      <c r="D22" s="24">
+      <c r="D22" s="14">
         <v>2352</v>
       </c>
-      <c r="E22" s="24">
+      <c r="E22" s="14">
         <v>1901</v>
       </c>
-      <c r="F22" s="24">
+      <c r="F22" s="14">
         <v>451</v>
       </c>
     </row>
     <row r="23" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="20" t="s">
+      <c r="B23" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C23" s="23">
+      <c r="C23" s="13">
         <v>2023</v>
       </c>
-      <c r="D23" s="24">
+      <c r="D23" s="14">
         <v>3543</v>
       </c>
-      <c r="E23" s="24">
+      <c r="E23" s="14">
         <v>2078</v>
       </c>
-      <c r="F23" s="24">
+      <c r="F23" s="14">
         <v>1465</v>
       </c>
     </row>
-    <row r="24" spans="2:6" s="22" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="21" t="s">
+    <row r="24" spans="2:6" s="12" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C24" s="25">
+      <c r="C24" s="15">
         <v>2023</v>
       </c>
-      <c r="D24" s="26">
+      <c r="D24" s="16">
         <v>76856</v>
       </c>
-      <c r="E24" s="26">
+      <c r="E24" s="16">
         <v>68374</v>
       </c>
-      <c r="F24" s="26">
+      <c r="F24" s="16">
         <v>8482</v>
       </c>
     </row>
     <row r="25" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="20" t="s">
+      <c r="B25" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C25" s="23">
+      <c r="C25" s="13">
         <v>2022</v>
       </c>
-      <c r="D25" s="24">
+      <c r="D25" s="14">
         <v>24810</v>
       </c>
-      <c r="E25" s="24">
+      <c r="E25" s="14">
         <v>23983</v>
       </c>
-      <c r="F25" s="24">
+      <c r="F25" s="14">
         <v>827</v>
       </c>
     </row>
     <row r="26" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="20" t="s">
+      <c r="B26" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C26" s="23">
+      <c r="C26" s="13">
         <v>2022</v>
       </c>
-      <c r="D26" s="24">
+      <c r="D26" s="14">
         <v>2289</v>
       </c>
-      <c r="E26" s="24">
+      <c r="E26" s="14">
         <v>2102</v>
       </c>
-      <c r="F26" s="24">
+      <c r="F26" s="14">
         <v>187</v>
       </c>
     </row>
     <row r="27" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="20" t="s">
+      <c r="B27" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C27" s="23">
+      <c r="C27" s="13">
         <v>2022</v>
       </c>
-      <c r="D27" s="24">
+      <c r="D27" s="14">
         <v>33410</v>
       </c>
-      <c r="E27" s="24">
+      <c r="E27" s="14">
         <v>30088</v>
       </c>
-      <c r="F27" s="24">
+      <c r="F27" s="14">
         <v>3322</v>
       </c>
     </row>
     <row r="28" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="20" t="s">
+      <c r="B28" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C28" s="23">
+      <c r="C28" s="13">
         <v>2022</v>
       </c>
-      <c r="D28" s="24">
+      <c r="D28" s="14">
         <v>10646</v>
       </c>
-      <c r="E28" s="24">
+      <c r="E28" s="14">
         <v>8761</v>
       </c>
-      <c r="F28" s="24">
+      <c r="F28" s="14">
         <v>1885</v>
       </c>
     </row>
     <row r="29" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="20" t="s">
+      <c r="B29" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C29" s="23">
+      <c r="C29" s="13">
         <v>2022</v>
       </c>
-      <c r="D29" s="24">
+      <c r="D29" s="14">
         <v>2228</v>
       </c>
-      <c r="E29" s="24">
+      <c r="E29" s="14">
         <v>1821</v>
       </c>
-      <c r="F29" s="24">
+      <c r="F29" s="14">
         <v>407</v>
       </c>
     </row>
     <row r="30" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="20" t="s">
+      <c r="B30" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C30" s="23">
+      <c r="C30" s="13">
         <v>2022</v>
       </c>
-      <c r="D30" s="24">
+      <c r="D30" s="14">
         <v>2858</v>
       </c>
-      <c r="E30" s="24">
+      <c r="E30" s="14">
         <v>1818</v>
       </c>
-      <c r="F30" s="24">
+      <c r="F30" s="14">
         <v>1040</v>
       </c>
     </row>
-    <row r="31" spans="2:6" s="22" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="21" t="s">
+    <row r="31" spans="2:6" s="12" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C31" s="25">
+      <c r="C31" s="15">
         <v>2022</v>
       </c>
-      <c r="D31" s="26">
+      <c r="D31" s="16">
         <v>76241</v>
       </c>
-      <c r="E31" s="26">
+      <c r="E31" s="16">
         <v>68573</v>
       </c>
-      <c r="F31" s="26">
+      <c r="F31" s="16">
         <v>7668</v>
       </c>
     </row>
     <row r="32" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="20" t="s">
+      <c r="B32" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C32" s="23">
+      <c r="C32" s="13">
         <v>2021</v>
       </c>
-      <c r="D32" s="24">
+      <c r="D32" s="14">
         <v>25484</v>
       </c>
-      <c r="E32" s="24">
+      <c r="E32" s="14">
         <v>24894</v>
       </c>
-      <c r="F32" s="24">
+      <c r="F32" s="14">
         <v>590</v>
       </c>
     </row>
     <row r="33" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="20" t="s">
+      <c r="B33" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C33" s="23">
+      <c r="C33" s="13">
         <v>2021</v>
       </c>
-      <c r="D33" s="24">
+      <c r="D33" s="14">
         <v>1997</v>
       </c>
-      <c r="E33" s="24">
+      <c r="E33" s="14">
         <v>1866</v>
       </c>
-      <c r="F33" s="24">
+      <c r="F33" s="14">
         <v>131</v>
       </c>
     </row>
     <row r="34" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="20" t="s">
+      <c r="B34" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C34" s="23">
+      <c r="C34" s="13">
         <v>2021</v>
       </c>
-      <c r="D34" s="24">
+      <c r="D34" s="14">
         <v>33930</v>
       </c>
-      <c r="E34" s="24">
+      <c r="E34" s="14">
         <v>30950</v>
       </c>
-      <c r="F34" s="24">
+      <c r="F34" s="14">
         <v>2980</v>
       </c>
     </row>
     <row r="35" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="20" t="s">
+      <c r="B35" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C35" s="23">
+      <c r="C35" s="13">
         <v>2021</v>
       </c>
-      <c r="D35" s="24">
+      <c r="D35" s="14">
         <v>10318</v>
       </c>
-      <c r="E35" s="24">
+      <c r="E35" s="14">
         <v>8716</v>
       </c>
-      <c r="F35" s="24">
+      <c r="F35" s="14">
         <v>1602</v>
       </c>
     </row>
     <row r="36" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="20" t="s">
+      <c r="B36" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C36" s="23">
+      <c r="C36" s="13">
         <v>2021</v>
       </c>
-      <c r="D36" s="24">
+      <c r="D36" s="14">
         <v>2188</v>
       </c>
-      <c r="E36" s="24">
+      <c r="E36" s="14">
         <v>1828</v>
       </c>
-      <c r="F36" s="24">
+      <c r="F36" s="14">
         <v>360</v>
       </c>
     </row>
     <row r="37" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="20" t="s">
+      <c r="B37" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C37" s="23">
+      <c r="C37" s="13">
         <v>2021</v>
       </c>
-      <c r="D37" s="24">
+      <c r="D37" s="14">
         <v>2402</v>
       </c>
-      <c r="E37" s="24">
+      <c r="E37" s="14">
         <v>1548</v>
       </c>
-      <c r="F37" s="24">
+      <c r="F37" s="14">
         <v>854</v>
       </c>
     </row>
-    <row r="38" spans="2:6" s="22" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="21" t="s">
+    <row r="38" spans="2:6" s="12" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C38" s="25">
+      <c r="C38" s="15">
         <v>2021</v>
       </c>
-      <c r="D38" s="26">
+      <c r="D38" s="16">
         <v>76319</v>
       </c>
-      <c r="E38" s="26">
+      <c r="E38" s="16">
         <v>69802</v>
       </c>
-      <c r="F38" s="26">
+      <c r="F38" s="16">
         <v>6517</v>
       </c>
     </row>
     <row r="39" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="20" t="s">
+      <c r="B39" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C39" s="23">
+      <c r="C39" s="13">
         <v>2020</v>
       </c>
-      <c r="D39" s="24">
+      <c r="D39" s="14">
         <v>5198</v>
       </c>
-      <c r="E39" s="24">
+      <c r="E39" s="14">
         <v>5039</v>
       </c>
-      <c r="F39" s="24">
+      <c r="F39" s="14">
         <v>159</v>
       </c>
     </row>
     <row r="40" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="20" t="s">
+      <c r="B40" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C40" s="23">
+      <c r="C40" s="13">
         <v>2020</v>
       </c>
-      <c r="D40" s="24">
+      <c r="D40" s="14">
         <v>1693</v>
       </c>
-      <c r="E40" s="24">
+      <c r="E40" s="14">
         <v>1592</v>
       </c>
-      <c r="F40" s="24">
+      <c r="F40" s="14">
         <v>101</v>
       </c>
     </row>
     <row r="41" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B41" s="20" t="s">
+      <c r="B41" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C41" s="23">
+      <c r="C41" s="13">
         <v>2020</v>
       </c>
-      <c r="D41" s="24">
+      <c r="D41" s="14">
         <v>35249</v>
       </c>
-      <c r="E41" s="24">
+      <c r="E41" s="14">
         <v>32466</v>
       </c>
-      <c r="F41" s="24">
+      <c r="F41" s="14">
         <v>2783</v>
       </c>
     </row>
     <row r="42" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="20" t="s">
+      <c r="B42" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C42" s="23">
+      <c r="C42" s="13">
         <v>2020</v>
       </c>
-      <c r="D42" s="24">
+      <c r="D42" s="14">
         <v>10566</v>
       </c>
-      <c r="E42" s="24">
+      <c r="E42" s="14">
         <v>8882</v>
       </c>
-      <c r="F42" s="24">
+      <c r="F42" s="14">
         <v>1684</v>
       </c>
     </row>
     <row r="43" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="20" t="s">
+      <c r="B43" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C43" s="23">
+      <c r="C43" s="13">
         <v>2020</v>
       </c>
-      <c r="D43" s="24">
+      <c r="D43" s="14">
         <v>2157</v>
       </c>
-      <c r="E43" s="24">
+      <c r="E43" s="14">
         <v>1853</v>
       </c>
-      <c r="F43" s="24">
+      <c r="F43" s="14">
         <v>304</v>
       </c>
     </row>
     <row r="44" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="20" t="s">
+      <c r="B44" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C44" s="23">
+      <c r="C44" s="13">
         <v>2020</v>
       </c>
-      <c r="D44" s="24">
+      <c r="D44" s="14">
         <v>2455</v>
       </c>
-      <c r="E44" s="24">
+      <c r="E44" s="14">
         <v>1543</v>
       </c>
-      <c r="F44" s="24">
+      <c r="F44" s="14">
         <v>912</v>
       </c>
     </row>
-    <row r="45" spans="2:6" s="22" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B45" s="21" t="s">
+    <row r="45" spans="2:6" s="12" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B45" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C45" s="25">
+      <c r="C45" s="15">
         <v>2020</v>
       </c>
-      <c r="D45" s="26">
+      <c r="D45" s="16">
         <v>57318</v>
       </c>
-      <c r="E45" s="26">
+      <c r="E45" s="16">
         <v>51375</v>
       </c>
-      <c r="F45" s="26">
+      <c r="F45" s="16">
         <v>5943</v>
       </c>
     </row>
     <row r="46" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="20" t="s">
+      <c r="B46" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C46" s="23">
+      <c r="C46" s="13">
         <v>2019</v>
       </c>
-      <c r="D46" s="27">
+      <c r="D46" s="17">
         <v>27080</v>
       </c>
-      <c r="E46" s="27">
+      <c r="E46" s="17">
         <v>26426</v>
       </c>
-      <c r="F46" s="27">
+      <c r="F46" s="17">
         <v>654</v>
       </c>
     </row>
     <row r="47" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="20" t="s">
+      <c r="B47" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C47" s="23">
+      <c r="C47" s="13">
         <v>2019</v>
       </c>
-      <c r="D47" s="27">
+      <c r="D47" s="17">
         <v>2350</v>
       </c>
-      <c r="E47" s="27">
+      <c r="E47" s="17">
         <v>2205</v>
       </c>
-      <c r="F47" s="27">
+      <c r="F47" s="17">
         <v>145</v>
       </c>
     </row>
     <row r="48" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="20" t="s">
+      <c r="B48" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C48" s="23">
+      <c r="C48" s="13">
         <v>2019</v>
       </c>
-      <c r="D48" s="27">
+      <c r="D48" s="17">
         <v>34113</v>
       </c>
-      <c r="E48" s="27">
+      <c r="E48" s="17">
         <v>31449</v>
       </c>
-      <c r="F48" s="27">
+      <c r="F48" s="17">
         <v>2664</v>
       </c>
     </row>
     <row r="49" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="20" t="s">
+      <c r="B49" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C49" s="23">
+      <c r="C49" s="13">
         <v>2019</v>
       </c>
-      <c r="D49" s="27">
+      <c r="D49" s="17">
         <v>11205</v>
       </c>
-      <c r="E49" s="27">
+      <c r="E49" s="17">
         <v>9629</v>
       </c>
-      <c r="F49" s="27">
+      <c r="F49" s="17">
         <v>1576</v>
       </c>
     </row>
     <row r="50" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="20" t="s">
+      <c r="B50" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C50" s="23">
+      <c r="C50" s="13">
         <v>2019</v>
       </c>
-      <c r="D50" s="27">
+      <c r="D50" s="17">
         <v>2067</v>
       </c>
-      <c r="E50" s="27">
+      <c r="E50" s="17">
         <v>1832</v>
       </c>
-      <c r="F50" s="27">
+      <c r="F50" s="17">
         <v>235</v>
       </c>
     </row>
     <row r="51" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="20" t="s">
+      <c r="B51" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C51" s="23">
+      <c r="C51" s="13">
         <v>2019</v>
       </c>
-      <c r="D51" s="27">
+      <c r="D51" s="17">
         <v>3357</v>
       </c>
-      <c r="E51" s="27">
+      <c r="E51" s="17">
         <v>2076</v>
       </c>
-      <c r="F51" s="27">
+      <c r="F51" s="17">
         <v>1281</v>
       </c>
-      <c r="G51" s="28"/>
-    </row>
-    <row r="52" spans="2:15" s="22" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="21" t="s">
+      <c r="G51" s="18"/>
+    </row>
+    <row r="52" spans="2:15" s="12" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B52" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C52" s="21">
+      <c r="C52" s="11">
         <v>2019</v>
       </c>
-      <c r="D52" s="29">
+      <c r="D52" s="19">
         <v>80172</v>
       </c>
-      <c r="E52" s="29">
+      <c r="E52" s="19">
         <v>73617</v>
       </c>
-      <c r="F52" s="29">
+      <c r="F52" s="19">
         <v>6555</v>
       </c>
-      <c r="G52" s="30"/>
+      <c r="G52" s="20"/>
     </row>
     <row r="53" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="20" t="s">
+      <c r="B53" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C53" s="23">
+      <c r="C53" s="13">
         <v>2018</v>
       </c>
-      <c r="D53" s="31">
+      <c r="D53" s="21">
         <v>26523</v>
       </c>
-      <c r="E53" s="32">
+      <c r="E53" s="22">
         <v>25872</v>
       </c>
-      <c r="F53" s="32">
+      <c r="F53" s="22">
         <v>651</v>
       </c>
     </row>
     <row r="54" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="20" t="s">
+      <c r="B54" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C54" s="23">
+      <c r="C54" s="13">
         <v>2018</v>
       </c>
-      <c r="D54" s="31">
+      <c r="D54" s="21">
         <v>2341</v>
       </c>
-      <c r="E54" s="32">
+      <c r="E54" s="22">
         <v>2216</v>
       </c>
-      <c r="F54" s="32">
+      <c r="F54" s="22">
         <v>125</v>
       </c>
     </row>
     <row r="55" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="20" t="s">
+      <c r="B55" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C55" s="23">
+      <c r="C55" s="13">
         <v>2018</v>
       </c>
-      <c r="D55" s="31">
+      <c r="D55" s="21">
         <v>35591</v>
       </c>
-      <c r="E55" s="32">
+      <c r="E55" s="22">
         <v>33213</v>
       </c>
-      <c r="F55" s="32">
+      <c r="F55" s="22">
         <v>2378</v>
       </c>
     </row>
     <row r="56" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B56" s="20" t="s">
+      <c r="B56" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C56" s="23">
+      <c r="C56" s="13">
         <v>2018</v>
       </c>
-      <c r="D56" s="31">
+      <c r="D56" s="21">
         <v>11516</v>
       </c>
-      <c r="E56" s="31">
+      <c r="E56" s="21">
         <v>9853</v>
       </c>
-      <c r="F56" s="31">
+      <c r="F56" s="21">
         <v>1663</v>
       </c>
     </row>
     <row r="57" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B57" s="20" t="s">
+      <c r="B57" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C57" s="23">
+      <c r="C57" s="13">
         <v>2018</v>
       </c>
-      <c r="D57" s="31">
+      <c r="D57" s="21">
         <v>1963</v>
       </c>
-      <c r="E57" s="32">
+      <c r="E57" s="22">
         <v>1751</v>
       </c>
-      <c r="F57" s="32">
+      <c r="F57" s="22">
         <v>212</v>
       </c>
     </row>
     <row r="58" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B58" s="20" t="s">
+      <c r="B58" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C58" s="23">
+      <c r="C58" s="13">
         <v>2018</v>
       </c>
-      <c r="D58" s="31">
+      <c r="D58" s="21">
         <v>3130</v>
       </c>
-      <c r="E58" s="32">
+      <c r="E58" s="22">
         <v>1915</v>
       </c>
-      <c r="F58" s="32">
+      <c r="F58" s="22">
         <v>1215</v>
       </c>
     </row>
-    <row r="59" spans="2:15" s="33" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B59" s="21" t="s">
+    <row r="59" spans="2:15" s="23" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B59" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C59" s="25">
+      <c r="C59" s="15">
         <v>2018</v>
       </c>
-      <c r="D59" s="27">
+      <c r="D59" s="17">
         <v>81064</v>
       </c>
-      <c r="E59" s="27">
+      <c r="E59" s="17">
         <v>74820</v>
       </c>
-      <c r="F59" s="27">
+      <c r="F59" s="17">
         <v>6244</v>
       </c>
     </row>
     <row r="60" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B60" s="20" t="s">
+      <c r="B60" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C60" s="23">
+      <c r="C60" s="13">
         <v>2017</v>
       </c>
-      <c r="D60" s="27">
+      <c r="D60" s="17">
         <v>26734</v>
       </c>
-      <c r="E60" s="27">
+      <c r="E60" s="17">
         <v>26092</v>
       </c>
-      <c r="F60" s="27">
+      <c r="F60" s="17">
         <v>642</v>
       </c>
-      <c r="G60" s="34"/>
-      <c r="H60" s="34"/>
-      <c r="I60" s="34"/>
-      <c r="L60" s="34"/>
-      <c r="M60" s="34"/>
-      <c r="N60" s="34"/>
-      <c r="O60" s="34"/>
+      <c r="G60" s="24"/>
+      <c r="H60" s="24"/>
+      <c r="I60" s="24"/>
+      <c r="L60" s="24"/>
+      <c r="M60" s="24"/>
+      <c r="N60" s="24"/>
+      <c r="O60" s="24"/>
     </row>
     <row r="61" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B61" s="20" t="s">
+      <c r="B61" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C61" s="23">
+      <c r="C61" s="13">
         <v>2017</v>
       </c>
-      <c r="D61" s="27">
+      <c r="D61" s="17">
         <v>2183</v>
       </c>
-      <c r="E61" s="27">
+      <c r="E61" s="17">
         <v>2019</v>
       </c>
-      <c r="F61" s="27">
+      <c r="F61" s="17">
         <v>164</v>
       </c>
-      <c r="G61" s="34"/>
-      <c r="H61" s="34"/>
-      <c r="I61" s="34"/>
-      <c r="L61" s="34"/>
-      <c r="M61" s="34"/>
-      <c r="N61" s="34"/>
-      <c r="O61" s="34"/>
+      <c r="G61" s="24"/>
+      <c r="H61" s="24"/>
+      <c r="I61" s="24"/>
+      <c r="L61" s="24"/>
+      <c r="M61" s="24"/>
+      <c r="N61" s="24"/>
+      <c r="O61" s="24"/>
     </row>
     <row r="62" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B62" s="20" t="s">
+      <c r="B62" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C62" s="23">
+      <c r="C62" s="13">
         <v>2017</v>
       </c>
-      <c r="D62" s="27">
+      <c r="D62" s="17">
         <v>37000</v>
       </c>
-      <c r="E62" s="27">
+      <c r="E62" s="17">
         <v>34782</v>
       </c>
-      <c r="F62" s="27">
+      <c r="F62" s="17">
         <v>2218</v>
       </c>
-      <c r="G62" s="34"/>
-      <c r="H62" s="34"/>
-      <c r="I62" s="34"/>
-      <c r="L62" s="34"/>
-      <c r="M62" s="34"/>
-      <c r="N62" s="34"/>
-      <c r="O62" s="34"/>
+      <c r="G62" s="24"/>
+      <c r="H62" s="24"/>
+      <c r="I62" s="24"/>
+      <c r="L62" s="24"/>
+      <c r="M62" s="24"/>
+      <c r="N62" s="24"/>
+      <c r="O62" s="24"/>
     </row>
     <row r="63" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B63" s="20" t="s">
+      <c r="B63" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C63" s="23">
+      <c r="C63" s="13">
         <v>2017</v>
       </c>
-      <c r="D63" s="27">
+      <c r="D63" s="17">
         <v>11686</v>
       </c>
-      <c r="E63" s="27">
+      <c r="E63" s="17">
         <v>10305</v>
       </c>
-      <c r="F63" s="27">
+      <c r="F63" s="17">
         <v>1381</v>
       </c>
-      <c r="G63" s="34"/>
-      <c r="H63" s="34"/>
-      <c r="I63" s="34"/>
-      <c r="L63" s="34"/>
-      <c r="M63" s="34"/>
-      <c r="N63" s="34"/>
-      <c r="O63" s="34"/>
+      <c r="G63" s="24"/>
+      <c r="H63" s="24"/>
+      <c r="I63" s="24"/>
+      <c r="L63" s="24"/>
+      <c r="M63" s="24"/>
+      <c r="N63" s="24"/>
+      <c r="O63" s="24"/>
     </row>
     <row r="64" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B64" s="20" t="s">
+      <c r="B64" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C64" s="23">
+      <c r="C64" s="13">
         <v>2017</v>
       </c>
-      <c r="D64" s="27">
+      <c r="D64" s="17">
         <v>1692</v>
       </c>
-      <c r="E64" s="27">
+      <c r="E64" s="17">
         <v>1507</v>
       </c>
-      <c r="F64" s="27">
+      <c r="F64" s="17">
         <v>185</v>
       </c>
-      <c r="G64" s="34"/>
-      <c r="H64" s="34"/>
-      <c r="I64" s="34"/>
-      <c r="L64" s="34"/>
-      <c r="M64" s="34"/>
-      <c r="N64" s="34"/>
-      <c r="O64" s="34"/>
+      <c r="G64" s="24"/>
+      <c r="H64" s="24"/>
+      <c r="I64" s="24"/>
+      <c r="L64" s="24"/>
+      <c r="M64" s="24"/>
+      <c r="N64" s="24"/>
+      <c r="O64" s="24"/>
     </row>
     <row r="65" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B65" s="20" t="s">
+      <c r="B65" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C65" s="23">
+      <c r="C65" s="13">
         <v>2017</v>
       </c>
-      <c r="D65" s="29">
+      <c r="D65" s="19">
         <v>3138</v>
       </c>
-      <c r="E65" s="29">
+      <c r="E65" s="19">
         <v>2013</v>
       </c>
-      <c r="F65" s="29">
+      <c r="F65" s="19">
         <v>1125</v>
       </c>
-      <c r="G65" s="34"/>
-      <c r="H65" s="34"/>
-      <c r="I65" s="34"/>
-      <c r="L65" s="34"/>
-      <c r="M65" s="34"/>
-      <c r="N65" s="34"/>
-      <c r="O65" s="34"/>
-    </row>
-    <row r="66" spans="2:15" s="22" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B66" s="21" t="s">
+      <c r="G65" s="24"/>
+      <c r="H65" s="24"/>
+      <c r="I65" s="24"/>
+      <c r="L65" s="24"/>
+      <c r="M65" s="24"/>
+      <c r="N65" s="24"/>
+      <c r="O65" s="24"/>
+    </row>
+    <row r="66" spans="2:15" s="12" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B66" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C66" s="25">
+      <c r="C66" s="15">
         <v>2017</v>
       </c>
-      <c r="D66" s="29">
+      <c r="D66" s="19">
         <v>82433</v>
       </c>
-      <c r="E66" s="29">
+      <c r="E66" s="19">
         <v>76718</v>
       </c>
-      <c r="F66" s="29">
+      <c r="F66" s="19">
         <v>5715</v>
       </c>
-      <c r="G66" s="35"/>
-      <c r="H66" s="35"/>
-      <c r="I66" s="35"/>
-      <c r="L66" s="35"/>
-      <c r="M66" s="35"/>
-      <c r="N66" s="35"/>
-      <c r="O66" s="35"/>
+      <c r="G66" s="25"/>
+      <c r="H66" s="25"/>
+      <c r="I66" s="25"/>
+      <c r="L66" s="25"/>
+      <c r="M66" s="25"/>
+      <c r="N66" s="25"/>
+      <c r="O66" s="25"/>
     </row>
     <row r="67" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B67" s="20" t="s">
+      <c r="B67" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C67" s="23">
+      <c r="C67" s="13">
         <v>2016</v>
       </c>
-      <c r="D67" s="27">
+      <c r="D67" s="17">
         <v>27554</v>
       </c>
-      <c r="E67" s="27">
+      <c r="E67" s="17">
         <v>26873</v>
       </c>
-      <c r="F67" s="27">
+      <c r="F67" s="17">
         <v>681</v>
       </c>
-      <c r="G67" s="34"/>
-      <c r="H67" s="34"/>
-      <c r="I67" s="34"/>
-      <c r="L67" s="34"/>
-      <c r="M67" s="34"/>
-      <c r="N67" s="34"/>
-      <c r="O67" s="34"/>
+      <c r="G67" s="24"/>
+      <c r="H67" s="24"/>
+      <c r="I67" s="24"/>
+      <c r="L67" s="24"/>
+      <c r="M67" s="24"/>
+      <c r="N67" s="24"/>
+      <c r="O67" s="24"/>
     </row>
     <row r="68" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B68" s="20" t="s">
+      <c r="B68" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C68" s="23">
+      <c r="C68" s="13">
         <v>2016</v>
       </c>
-      <c r="D68" s="27">
+      <c r="D68" s="17">
         <v>1918</v>
       </c>
-      <c r="E68" s="27">
+      <c r="E68" s="17">
         <v>1802</v>
       </c>
-      <c r="F68" s="27">
+      <c r="F68" s="17">
         <v>116</v>
       </c>
-      <c r="G68" s="36"/>
-      <c r="H68" s="36"/>
-      <c r="I68" s="36"/>
-      <c r="L68" s="36"/>
-      <c r="M68" s="36"/>
-      <c r="N68" s="36"/>
-      <c r="O68" s="36"/>
+      <c r="G68" s="26"/>
+      <c r="H68" s="26"/>
+      <c r="I68" s="26"/>
+      <c r="L68" s="26"/>
+      <c r="M68" s="26"/>
+      <c r="N68" s="26"/>
+      <c r="O68" s="26"/>
     </row>
     <row r="69" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B69" s="20" t="s">
+      <c r="B69" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C69" s="23">
+      <c r="C69" s="13">
         <v>2016</v>
       </c>
-      <c r="D69" s="27">
+      <c r="D69" s="17">
         <v>39059</v>
       </c>
-      <c r="E69" s="27">
+      <c r="E69" s="17">
         <v>36674</v>
       </c>
-      <c r="F69" s="27">
+      <c r="F69" s="17">
         <v>2385</v>
       </c>
     </row>
     <row r="70" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B70" s="20" t="s">
+      <c r="B70" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C70" s="23">
+      <c r="C70" s="13">
         <v>2016</v>
       </c>
-      <c r="D70" s="27">
+      <c r="D70" s="17">
         <v>11333</v>
       </c>
-      <c r="E70" s="27">
+      <c r="E70" s="17">
         <v>10096</v>
       </c>
-      <c r="F70" s="27">
+      <c r="F70" s="17">
         <v>1237</v>
       </c>
     </row>
     <row r="71" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B71" s="20" t="s">
+      <c r="B71" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C71" s="23">
+      <c r="C71" s="13">
         <v>2016</v>
       </c>
-      <c r="D71" s="27">
+      <c r="D71" s="17">
         <v>1780</v>
       </c>
-      <c r="E71" s="27">
+      <c r="E71" s="17">
         <v>1582</v>
       </c>
-      <c r="F71" s="27">
+      <c r="F71" s="17">
         <v>198</v>
       </c>
     </row>
     <row r="72" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B72" s="20" t="s">
+      <c r="B72" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C72" s="23">
+      <c r="C72" s="13">
         <v>2016</v>
       </c>
-      <c r="D72" s="27">
+      <c r="D72" s="17">
         <v>2511</v>
       </c>
-      <c r="E72" s="27">
+      <c r="E72" s="17">
         <v>1849</v>
       </c>
-      <c r="F72" s="27">
+      <c r="F72" s="17">
         <v>662</v>
       </c>
     </row>
-    <row r="73" spans="2:15" s="22" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B73" s="21" t="s">
+    <row r="73" spans="2:15" s="12" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B73" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C73" s="25">
+      <c r="C73" s="15">
         <v>2016</v>
       </c>
-      <c r="D73" s="29">
+      <c r="D73" s="19">
         <v>84155</v>
       </c>
-      <c r="E73" s="29">
+      <c r="E73" s="19">
         <v>78876</v>
       </c>
-      <c r="F73" s="29">
+      <c r="F73" s="19">
         <v>5279</v>
       </c>
     </row>
     <row r="74" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B74" s="20" t="s">
+      <c r="B74" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C74" s="23">
+      <c r="C74" s="13">
         <v>2015</v>
       </c>
-      <c r="D74" s="27">
+      <c r="D74" s="17">
         <v>27892</v>
       </c>
-      <c r="E74" s="27">
+      <c r="E74" s="17">
         <v>27241</v>
       </c>
-      <c r="F74" s="27">
+      <c r="F74" s="17">
         <v>651</v>
       </c>
     </row>
     <row r="75" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B75" s="20" t="s">
+      <c r="B75" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C75" s="23">
+      <c r="C75" s="13">
         <v>2015</v>
       </c>
-      <c r="D75" s="27">
+      <c r="D75" s="17">
         <v>1797</v>
       </c>
-      <c r="E75" s="27">
+      <c r="E75" s="17">
         <v>1663</v>
       </c>
-      <c r="F75" s="27">
+      <c r="F75" s="17">
         <v>134</v>
       </c>
     </row>
     <row r="76" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B76" s="20" t="s">
+      <c r="B76" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C76" s="23">
+      <c r="C76" s="13">
         <v>2015</v>
       </c>
-      <c r="D76" s="27">
+      <c r="D76" s="17">
         <v>40641</v>
       </c>
-      <c r="E76" s="27">
+      <c r="E76" s="17">
         <v>37907</v>
       </c>
-      <c r="F76" s="27">
+      <c r="F76" s="17">
         <v>2734</v>
       </c>
     </row>
     <row r="77" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B77" s="20" t="s">
+      <c r="B77" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C77" s="23">
+      <c r="C77" s="13">
         <v>2015</v>
       </c>
-      <c r="D77" s="27">
+      <c r="D77" s="17">
         <v>11120</v>
       </c>
-      <c r="E77" s="27">
+      <c r="E77" s="17">
         <v>9873</v>
       </c>
-      <c r="F77" s="27">
+      <c r="F77" s="17">
         <v>1247</v>
       </c>
     </row>
     <row r="78" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B78" s="20" t="s">
+      <c r="B78" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C78" s="23">
+      <c r="C78" s="13">
         <v>2015</v>
       </c>
-      <c r="D78" s="27">
+      <c r="D78" s="17">
         <v>2007</v>
       </c>
-      <c r="E78" s="27">
+      <c r="E78" s="17">
         <v>1727</v>
       </c>
-      <c r="F78" s="27">
+      <c r="F78" s="17">
         <v>280</v>
       </c>
     </row>
     <row r="79" spans="2:15" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B79" s="20" t="s">
+      <c r="B79" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C79" s="23">
+      <c r="C79" s="13">
         <v>2015</v>
       </c>
-      <c r="D79" s="27">
+      <c r="D79" s="17">
         <v>2332</v>
       </c>
-      <c r="E79" s="27">
+      <c r="E79" s="17">
         <v>1809</v>
       </c>
-      <c r="F79" s="27">
+      <c r="F79" s="17">
         <v>523</v>
       </c>
     </row>
-    <row r="80" spans="2:15" s="22" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B80" s="21" t="s">
+    <row r="80" spans="2:15" s="12" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B80" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C80" s="25">
+      <c r="C80" s="15">
         <v>2015</v>
       </c>
-      <c r="D80" s="37">
+      <c r="D80" s="27">
         <v>85789</v>
       </c>
-      <c r="E80" s="29">
+      <c r="E80" s="19">
         <v>80220</v>
       </c>
-      <c r="F80" s="37">
+      <c r="F80" s="27">
         <v>5569</v>
       </c>
     </row>
     <row r="81" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B81" s="20" t="s">
+      <c r="B81" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C81" s="38">
+      <c r="C81" s="28">
         <v>2014</v>
       </c>
-      <c r="D81" s="39">
+      <c r="D81" s="29">
         <v>26724</v>
       </c>
-      <c r="E81" s="39">
+      <c r="E81" s="29">
         <v>26061</v>
       </c>
-      <c r="F81" s="39">
+      <c r="F81" s="29">
         <v>663</v>
       </c>
-      <c r="G81" s="40"/>
-      <c r="H81" s="40"/>
-      <c r="I81" s="40"/>
+      <c r="G81" s="30"/>
+      <c r="H81" s="30"/>
+      <c r="I81" s="30"/>
     </row>
     <row r="82" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B82" s="20" t="s">
+      <c r="B82" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C82" s="38">
+      <c r="C82" s="28">
         <v>2014</v>
       </c>
-      <c r="D82" s="39">
+      <c r="D82" s="29">
         <v>1839</v>
       </c>
-      <c r="E82" s="39">
+      <c r="E82" s="29">
         <v>1700</v>
       </c>
-      <c r="F82" s="39">
+      <c r="F82" s="29">
         <v>139</v>
       </c>
     </row>
     <row r="83" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B83" s="20" t="s">
+      <c r="B83" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C83" s="38">
+      <c r="C83" s="28">
         <v>2014</v>
       </c>
-      <c r="D83" s="39">
+      <c r="D83" s="29">
         <v>42449</v>
       </c>
-      <c r="E83" s="39">
+      <c r="E83" s="29">
         <v>39729</v>
       </c>
-      <c r="F83" s="39">
+      <c r="F83" s="29">
         <v>2720</v>
       </c>
     </row>
     <row r="84" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B84" s="20" t="s">
+      <c r="B84" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C84" s="38">
+      <c r="C84" s="28">
         <v>2014</v>
       </c>
-      <c r="D84" s="39">
+      <c r="D84" s="29">
         <v>12027</v>
       </c>
-      <c r="E84" s="39">
+      <c r="E84" s="29">
         <v>10816</v>
       </c>
-      <c r="F84" s="39">
+      <c r="F84" s="29">
         <v>1211</v>
       </c>
     </row>
     <row r="85" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B85" s="20" t="s">
+      <c r="B85" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C85" s="38">
+      <c r="C85" s="28">
         <v>2014</v>
       </c>
-      <c r="D85" s="39">
+      <c r="D85" s="29">
         <v>1964</v>
       </c>
-      <c r="E85" s="39">
+      <c r="E85" s="29">
         <v>1743</v>
       </c>
-      <c r="F85" s="39">
+      <c r="F85" s="29">
         <v>221</v>
       </c>
     </row>
     <row r="86" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B86" s="20" t="s">
+      <c r="B86" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C86" s="38">
+      <c r="C86" s="28">
         <v>2014</v>
       </c>
-      <c r="D86" s="39">
+      <c r="D86" s="29">
         <v>2281</v>
       </c>
-      <c r="E86" s="39">
+      <c r="E86" s="29">
         <v>1843</v>
       </c>
-      <c r="F86" s="39">
+      <c r="F86" s="29">
         <v>438</v>
       </c>
     </row>
-    <row r="87" spans="2:10" s="22" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B87" s="21" t="s">
+    <row r="87" spans="2:10" s="12" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B87" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C87" s="41">
+      <c r="C87" s="31">
         <v>2014</v>
       </c>
-      <c r="D87" s="42">
+      <c r="D87" s="32">
         <v>87284</v>
       </c>
-      <c r="E87" s="42">
+      <c r="E87" s="32">
         <v>81892</v>
       </c>
-      <c r="F87" s="42">
+      <c r="F87" s="32">
         <v>5392</v>
       </c>
     </row>
     <row r="88" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B88" s="20" t="s">
+      <c r="B88" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C88" s="43">
+      <c r="C88" s="33">
         <v>2013</v>
       </c>
-      <c r="D88" s="31">
+      <c r="D88" s="21">
         <v>25788</v>
       </c>
-      <c r="E88" s="32">
+      <c r="E88" s="22">
         <v>25264</v>
       </c>
-      <c r="F88" s="31">
+      <c r="F88" s="21">
         <v>524</v>
       </c>
-      <c r="J88" s="44" t="s">
+      <c r="J88" s="34" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="89" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B89" s="20" t="s">
+      <c r="B89" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C89" s="43">
+      <c r="C89" s="33">
         <v>2013</v>
       </c>
-      <c r="D89" s="31">
+      <c r="D89" s="21">
         <v>1963</v>
       </c>
-      <c r="E89" s="32">
+      <c r="E89" s="22">
         <v>1881</v>
       </c>
-      <c r="F89" s="31">
+      <c r="F89" s="21">
         <v>82</v>
       </c>
     </row>
     <row r="90" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B90" s="20" t="s">
+      <c r="B90" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C90" s="43">
+      <c r="C90" s="33">
         <v>2013</v>
       </c>
-      <c r="D90" s="31">
+      <c r="D90" s="21">
         <v>42205</v>
       </c>
-      <c r="E90" s="32">
+      <c r="E90" s="22">
         <v>39852</v>
       </c>
-      <c r="F90" s="31">
+      <c r="F90" s="21">
         <v>2353</v>
       </c>
     </row>
     <row r="91" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B91" s="20" t="s">
+      <c r="B91" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C91" s="43">
+      <c r="C91" s="33">
         <v>2013</v>
       </c>
-      <c r="D91" s="31">
+      <c r="D91" s="21">
         <v>12132</v>
       </c>
-      <c r="E91" s="32">
+      <c r="E91" s="22">
         <v>11000</v>
       </c>
-      <c r="F91" s="31">
+      <c r="F91" s="21">
         <v>1132</v>
       </c>
     </row>
     <row r="92" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B92" s="20" t="s">
+      <c r="B92" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C92" s="43">
+      <c r="C92" s="33">
         <v>2013</v>
       </c>
-      <c r="D92" s="31">
+      <c r="D92" s="21">
         <v>2002</v>
       </c>
-      <c r="E92" s="32">
+      <c r="E92" s="22">
         <v>1749</v>
       </c>
-      <c r="F92" s="31">
+      <c r="F92" s="21">
         <v>253</v>
       </c>
     </row>
     <row r="93" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B93" s="20" t="s">
+      <c r="B93" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C93" s="43">
+      <c r="C93" s="33">
         <v>2013</v>
       </c>
-      <c r="D93" s="31">
+      <c r="D93" s="21">
         <v>2370</v>
       </c>
-      <c r="E93" s="32">
+      <c r="E93" s="22">
         <v>1974</v>
       </c>
-      <c r="F93" s="31">
+      <c r="F93" s="21">
         <v>396</v>
       </c>
     </row>
-    <row r="94" spans="2:10" s="22" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B94" s="21" t="s">
+    <row r="94" spans="2:10" s="12" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B94" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C94" s="41">
+      <c r="C94" s="31">
         <v>2013</v>
       </c>
-      <c r="D94" s="37">
+      <c r="D94" s="27">
         <v>86460</v>
       </c>
-      <c r="E94" s="29">
+      <c r="E94" s="19">
         <v>81720</v>
       </c>
-      <c r="F94" s="37">
+      <c r="F94" s="27">
         <v>4740</v>
       </c>
     </row>
     <row r="95" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B95" s="45" t="s">
+      <c r="B95" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="C95" s="46">
+      <c r="C95" s="36">
         <v>2012</v>
       </c>
-      <c r="D95" s="32">
+      <c r="D95" s="22">
         <v>26655</v>
       </c>
-      <c r="E95" s="32">
+      <c r="E95" s="22">
         <v>25981</v>
       </c>
-      <c r="F95" s="32">
+      <c r="F95" s="22">
         <v>674</v>
       </c>
     </row>
     <row r="96" spans="2:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B96" s="20" t="s">
+      <c r="B96" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C96" s="38">
+      <c r="C96" s="28">
         <v>2012</v>
       </c>
-      <c r="D96" s="39">
+      <c r="D96" s="29">
         <v>1779</v>
       </c>
-      <c r="E96" s="39">
+      <c r="E96" s="29">
         <v>1673</v>
       </c>
-      <c r="F96" s="39">
+      <c r="F96" s="29">
         <v>106</v>
       </c>
     </row>
     <row r="97" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B97" s="20" t="s">
+      <c r="B97" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C97" s="38">
+      <c r="C97" s="28">
         <v>2012</v>
       </c>
-      <c r="D97" s="39">
+      <c r="D97" s="29">
         <v>41339</v>
       </c>
-      <c r="E97" s="39">
+      <c r="E97" s="29">
         <v>38964</v>
       </c>
-      <c r="F97" s="39">
+      <c r="F97" s="29">
         <v>2375</v>
       </c>
     </row>
     <row r="98" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B98" s="20" t="s">
+      <c r="B98" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C98" s="38">
+      <c r="C98" s="28">
         <v>2012</v>
       </c>
-      <c r="D98" s="39">
+      <c r="D98" s="29">
         <v>12870</v>
       </c>
-      <c r="E98" s="39">
+      <c r="E98" s="29">
         <v>11647</v>
       </c>
-      <c r="F98" s="39">
+      <c r="F98" s="29">
         <v>1223</v>
       </c>
     </row>
     <row r="99" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B99" s="20" t="s">
+      <c r="B99" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C99" s="38">
+      <c r="C99" s="28">
         <v>2012</v>
       </c>
-      <c r="D99" s="39">
+      <c r="D99" s="29">
         <v>2073</v>
       </c>
-      <c r="E99" s="39">
+      <c r="E99" s="29">
         <v>1875</v>
       </c>
-      <c r="F99" s="39">
+      <c r="F99" s="29">
         <v>198</v>
       </c>
     </row>
     <row r="100" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B100" s="20" t="s">
+      <c r="B100" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C100" s="38">
+      <c r="C100" s="28">
         <v>2012</v>
       </c>
-      <c r="D100" s="39">
+      <c r="D100" s="29">
         <v>2700</v>
       </c>
-      <c r="E100" s="39">
+      <c r="E100" s="29">
         <v>2207</v>
       </c>
-      <c r="F100" s="39">
+      <c r="F100" s="29">
         <v>493</v>
       </c>
     </row>
-    <row r="101" spans="2:6" s="22" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B101" s="21" t="s">
+    <row r="101" spans="2:6" s="12" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B101" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C101" s="41">
+      <c r="C101" s="31">
         <v>2012</v>
       </c>
-      <c r="D101" s="42">
+      <c r="D101" s="32">
         <v>87416</v>
       </c>
-      <c r="E101" s="42">
+      <c r="E101" s="32">
         <v>82347</v>
       </c>
-      <c r="F101" s="42">
+      <c r="F101" s="32">
         <v>5069</v>
       </c>
     </row>
     <row r="102" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B102" s="20" t="s">
+      <c r="B102" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C102" s="38">
+      <c r="C102" s="28">
         <v>2011</v>
       </c>
-      <c r="D102" s="39">
+      <c r="D102" s="29">
         <v>42076</v>
       </c>
-      <c r="E102" s="39">
+      <c r="E102" s="29">
         <v>41181</v>
       </c>
-      <c r="F102" s="39">
+      <c r="F102" s="29">
         <v>895</v>
       </c>
     </row>
     <row r="103" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B103" s="20" t="s">
+      <c r="B103" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C103" s="38">
+      <c r="C103" s="28">
         <v>2011</v>
       </c>
-      <c r="D103" s="39">
+      <c r="D103" s="29">
         <v>1547</v>
       </c>
-      <c r="E103" s="39">
+      <c r="E103" s="29">
         <v>1476</v>
       </c>
-      <c r="F103" s="39">
+      <c r="F103" s="29">
         <v>71</v>
       </c>
     </row>
     <row r="104" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B104" s="20" t="s">
+      <c r="B104" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C104" s="38">
+      <c r="C104" s="28">
         <v>2011</v>
       </c>
-      <c r="D104" s="39">
+      <c r="D104" s="29">
         <v>41338</v>
       </c>
-      <c r="E104" s="39">
+      <c r="E104" s="29">
         <v>39147</v>
       </c>
-      <c r="F104" s="39">
+      <c r="F104" s="29">
         <v>2191</v>
       </c>
     </row>
     <row r="105" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B105" s="20" t="s">
+      <c r="B105" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C105" s="38">
+      <c r="C105" s="28">
         <v>2011</v>
       </c>
-      <c r="D105" s="39">
+      <c r="D105" s="29">
         <v>12695</v>
       </c>
-      <c r="E105" s="39">
+      <c r="E105" s="29">
         <v>11563</v>
       </c>
-      <c r="F105" s="39">
+      <c r="F105" s="29">
         <v>1132</v>
       </c>
     </row>
     <row r="106" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B106" s="20" t="s">
+      <c r="B106" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C106" s="38">
+      <c r="C106" s="28">
         <v>2011</v>
       </c>
-      <c r="D106" s="39">
+      <c r="D106" s="29">
         <v>2267</v>
       </c>
-      <c r="E106" s="39">
+      <c r="E106" s="29">
         <v>1963</v>
       </c>
-      <c r="F106" s="39">
+      <c r="F106" s="29">
         <v>304</v>
       </c>
     </row>
     <row r="107" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B107" s="20" t="s">
+      <c r="B107" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C107" s="38">
+      <c r="C107" s="28">
         <v>2011</v>
       </c>
-      <c r="D107" s="39">
+      <c r="D107" s="29">
         <v>2818</v>
       </c>
-      <c r="E107" s="39">
+      <c r="E107" s="29">
         <v>2325</v>
       </c>
-      <c r="F107" s="39">
+      <c r="F107" s="29">
         <v>493</v>
       </c>
     </row>
-    <row r="108" spans="2:6" s="22" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B108" s="21" t="s">
+    <row r="108" spans="2:6" s="12" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B108" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C108" s="41">
+      <c r="C108" s="31">
         <v>2011</v>
       </c>
-      <c r="D108" s="42">
+      <c r="D108" s="32">
         <v>102741</v>
       </c>
-      <c r="E108" s="42">
+      <c r="E108" s="32">
         <v>97655</v>
       </c>
-      <c r="F108" s="42">
+      <c r="F108" s="32">
         <v>5086</v>
       </c>
     </row>
     <row r="109" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B109" s="45" t="s">
+      <c r="B109" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="C109" s="46">
+      <c r="C109" s="36">
         <v>2010</v>
       </c>
-      <c r="D109" s="32">
+      <c r="D109" s="22">
         <v>24950</v>
       </c>
-      <c r="E109" s="32">
+      <c r="E109" s="22">
         <v>24492</v>
       </c>
-      <c r="F109" s="32">
+      <c r="F109" s="22">
         <v>458</v>
       </c>
     </row>
     <row r="110" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B110" s="20" t="s">
+      <c r="B110" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C110" s="38">
+      <c r="C110" s="28">
         <v>2010</v>
       </c>
-      <c r="D110" s="39">
+      <c r="D110" s="29">
         <v>1346</v>
       </c>
-      <c r="E110" s="39">
+      <c r="E110" s="29">
         <v>1252</v>
       </c>
-      <c r="F110" s="39">
+      <c r="F110" s="29">
         <v>94</v>
       </c>
     </row>
     <row r="111" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B111" s="20" t="s">
+      <c r="B111" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C111" s="38">
+      <c r="C111" s="28">
         <v>2010</v>
       </c>
-      <c r="D111" s="39">
+      <c r="D111" s="29">
         <v>41347</v>
       </c>
-      <c r="E111" s="39">
+      <c r="E111" s="29">
         <v>38745</v>
       </c>
-      <c r="F111" s="39">
+      <c r="F111" s="29">
         <v>2602</v>
       </c>
     </row>
     <row r="112" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B112" s="20" t="s">
+      <c r="B112" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C112" s="38">
+      <c r="C112" s="28">
         <v>2010</v>
       </c>
-      <c r="D112" s="39">
+      <c r="D112" s="29">
         <v>14462</v>
       </c>
-      <c r="E112" s="39">
+      <c r="E112" s="29">
         <v>12814</v>
       </c>
-      <c r="F112" s="39">
+      <c r="F112" s="29">
         <v>1648</v>
       </c>
     </row>
     <row r="113" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B113" s="20" t="s">
+      <c r="B113" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C113" s="38">
+      <c r="C113" s="28">
         <v>2010</v>
       </c>
-      <c r="D113" s="39">
+      <c r="D113" s="29">
         <v>2153</v>
       </c>
-      <c r="E113" s="39">
+      <c r="E113" s="29">
         <v>1818</v>
       </c>
-      <c r="F113" s="39">
+      <c r="F113" s="29">
         <v>335</v>
       </c>
     </row>
     <row r="114" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B114" s="20" t="s">
+      <c r="B114" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C114" s="38">
+      <c r="C114" s="28">
         <v>2010</v>
       </c>
-      <c r="D114" s="39">
+      <c r="D114" s="29">
         <v>3065</v>
       </c>
-      <c r="E114" s="39">
+      <c r="E114" s="29">
         <v>2471</v>
       </c>
-      <c r="F114" s="39">
+      <c r="F114" s="29">
         <v>594</v>
       </c>
     </row>
-    <row r="115" spans="2:6" s="22" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B115" s="21" t="s">
+    <row r="115" spans="2:6" s="12" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B115" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C115" s="41">
+      <c r="C115" s="31">
         <v>2010</v>
       </c>
-      <c r="D115" s="42">
+      <c r="D115" s="32">
         <v>87323</v>
       </c>
-      <c r="E115" s="42">
+      <c r="E115" s="32">
         <v>81592</v>
       </c>
-      <c r="F115" s="42">
+      <c r="F115" s="32">
         <v>5731</v>
       </c>
     </row>
     <row r="116" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B116" s="45" t="s">
+      <c r="B116" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="C116" s="46">
+      <c r="C116" s="36">
         <v>2005</v>
       </c>
-      <c r="D116" s="32">
+      <c r="D116" s="22">
         <v>20073</v>
       </c>
-      <c r="E116" s="32">
+      <c r="E116" s="22">
         <v>19598</v>
       </c>
-      <c r="F116" s="32">
+      <c r="F116" s="22">
         <v>475</v>
       </c>
     </row>
     <row r="117" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B117" s="20" t="s">
+      <c r="B117" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C117" s="46">
+      <c r="C117" s="36">
         <v>2005</v>
       </c>
-      <c r="D117" s="27">
+      <c r="D117" s="17">
         <v>1757</v>
       </c>
-      <c r="E117" s="27">
+      <c r="E117" s="17">
         <v>1655</v>
       </c>
-      <c r="F117" s="27">
+      <c r="F117" s="17">
         <v>102</v>
       </c>
     </row>
     <row r="118" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B118" s="20" t="s">
+      <c r="B118" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C118" s="46">
+      <c r="C118" s="36">
         <v>2005</v>
       </c>
-      <c r="D118" s="27">
+      <c r="D118" s="17">
         <v>43181</v>
       </c>
-      <c r="E118" s="27">
+      <c r="E118" s="17">
         <v>40717</v>
       </c>
-      <c r="F118" s="27">
+      <c r="F118" s="17">
         <v>2464</v>
       </c>
     </row>
     <row r="119" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B119" s="20" t="s">
+      <c r="B119" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C119" s="46">
+      <c r="C119" s="36">
         <v>2005</v>
       </c>
-      <c r="D119" s="27">
+      <c r="D119" s="17">
         <v>18693</v>
       </c>
-      <c r="E119" s="27">
+      <c r="E119" s="17">
         <v>16919</v>
       </c>
-      <c r="F119" s="27">
+      <c r="F119" s="17">
         <v>1774</v>
       </c>
     </row>
     <row r="120" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B120" s="20" t="s">
+      <c r="B120" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C120" s="46">
+      <c r="C120" s="36">
         <v>2005</v>
       </c>
-      <c r="D120" s="27">
+      <c r="D120" s="17">
         <v>3384</v>
       </c>
-      <c r="E120" s="27">
+      <c r="E120" s="17">
         <v>2694</v>
       </c>
-      <c r="F120" s="27">
+      <c r="F120" s="17">
         <v>690</v>
       </c>
     </row>
     <row r="121" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B121" s="20" t="s">
+      <c r="B121" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C121" s="46">
+      <c r="C121" s="36">
         <v>2005</v>
       </c>
-      <c r="D121" s="27">
+      <c r="D121" s="17">
         <v>4961</v>
       </c>
-      <c r="E121" s="27">
+      <c r="E121" s="17">
         <v>4044</v>
       </c>
-      <c r="F121" s="27">
+      <c r="F121" s="17">
         <v>917</v>
       </c>
     </row>
-    <row r="122" spans="2:6" s="22" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B122" s="21" t="s">
+    <row r="122" spans="2:6" s="12" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B122" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C122" s="47">
+      <c r="C122" s="37">
         <v>2005</v>
       </c>
-      <c r="D122" s="29">
+      <c r="D122" s="19">
         <v>92049</v>
       </c>
-      <c r="E122" s="29">
+      <c r="E122" s="19">
         <v>85627</v>
       </c>
-      <c r="F122" s="29">
+      <c r="F122" s="19">
         <v>6422</v>
       </c>
     </row>
     <row r="123" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B123" s="48"/>
-      <c r="C123" s="49"/>
-      <c r="D123" s="50"/>
-      <c r="E123" s="51"/>
-      <c r="F123" s="51"/>
+      <c r="B123" s="38"/>
+      <c r="C123" s="39"/>
+      <c r="D123" s="40"/>
+      <c r="E123" s="41"/>
+      <c r="F123" s="41"/>
     </row>
     <row r="124" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B124" s="52" t="s">
+      <c r="B124" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="C124" s="53"/>
-      <c r="D124" s="50"/>
-      <c r="E124" s="51"/>
-      <c r="F124" s="51"/>
+      <c r="C124" s="43"/>
+      <c r="D124" s="40"/>
+      <c r="E124" s="41"/>
+      <c r="F124" s="41"/>
     </row>
     <row r="125" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B125" s="54" t="s">
+      <c r="B125" s="44" t="s">
         <v>22</v>
       </c>
-      <c r="C125" s="53"/>
-      <c r="D125" s="50"/>
-      <c r="E125" s="51"/>
-      <c r="F125" s="51"/>
+      <c r="C125" s="43"/>
+      <c r="D125" s="40"/>
+      <c r="E125" s="41"/>
+      <c r="F125" s="41"/>
     </row>
     <row r="126" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B126" s="54" t="s">
+      <c r="B126" s="44" t="s">
         <v>23</v>
       </c>
-      <c r="C126" s="53"/>
-      <c r="D126" s="50"/>
-      <c r="E126" s="51"/>
-      <c r="F126" s="51"/>
+      <c r="C126" s="43"/>
+      <c r="D126" s="40"/>
+      <c r="E126" s="41"/>
+      <c r="F126" s="41"/>
     </row>
     <row r="127" spans="2:6" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C127" s="55"/>
-      <c r="D127" s="50"/>
-      <c r="E127" s="51"/>
-      <c r="F127" s="51"/>
-    </row>
-    <row r="128" spans="2:6" s="56" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B128" s="57" t="s">
+      <c r="C127" s="45"/>
+      <c r="D127" s="40"/>
+      <c r="E127" s="41"/>
+      <c r="F127" s="41"/>
+    </row>
+    <row r="128" spans="2:6" s="46" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B128" s="47" t="s">
         <v>24</v>
       </c>
-      <c r="C128" s="55"/>
-      <c r="D128" s="58"/>
-      <c r="E128" s="59"/>
-      <c r="F128" s="59"/>
-    </row>
-    <row r="129" spans="2:3" s="56" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="C129" s="43"/>
-    </row>
-    <row r="130" spans="2:3" s="56" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B130" s="56" t="s">
+      <c r="C128" s="45"/>
+      <c r="D128" s="48"/>
+      <c r="E128" s="49"/>
+      <c r="F128" s="49"/>
+    </row>
+    <row r="129" spans="2:3" s="46" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="C129" s="33"/>
+    </row>
+    <row r="130" spans="2:3" s="46" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B130" s="46" t="s">
         <v>25</v>
       </c>
-      <c r="C130" s="43"/>
-    </row>
-    <row r="131" spans="2:3" s="56" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B131" s="56" t="s">
+      <c r="C130" s="33"/>
+    </row>
+    <row r="131" spans="2:3" s="46" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B131" s="46" t="s">
+        <v>28</v>
+      </c>
+      <c r="C131" s="33"/>
+    </row>
+    <row r="132" spans="2:3" s="46" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B132" s="46" t="s">
         <v>26</v>
       </c>
-      <c r="C131" s="43"/>
-    </row>
-    <row r="132" spans="2:3" s="56" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B132" s="56" t="s">
+      <c r="C132" s="33"/>
+    </row>
+    <row r="133" spans="2:3" s="46" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B133" s="50" t="s">
         <v>27</v>
       </c>
-      <c r="C132" s="43"/>
-    </row>
-    <row r="133" spans="2:3" s="56" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B133" s="60" t="s">
-        <v>28</v>
-      </c>
-      <c r="C133" s="43"/>
+      <c r="C133" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>